<commit_message>
Updated RBF - DS Telejan now has proper Mahjongg controls and Flying Ball is fixed
</commit_message>
<xml_diff>
--- a/Useful Information/DECO_Cassette_Test_List.xlsx
+++ b/Useful Information/DECO_Cassette_Test_List.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="142">
   <si>
     <t xml:space="preserve">Game Name</t>
   </si>
@@ -61,150 +61,141 @@
     <t xml:space="preserve">cprogolf18</t>
   </si>
   <si>
+    <t xml:space="preserve">Angler Dangler (DECO Cassette) (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cadanglr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Astro Fantasia (DECO Cassette) (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">castfant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boulder Dash (DECO Cassette) (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cbdash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bump 'n' Jump (DECO Cassette) (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cbnj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burger Time (DECO Cassette) (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cbtime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burnin' Rubber (DECO Cassette) (Japan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cburnrubj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burnin' Rubber (DECO Cassette)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cburnrub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burnin' Rubber (DECO Cassette) (US) (set 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cburnrub2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cluster Buster (DECO Cassette) (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cgraplop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECO Cassette System ROM Multigame (Darksoft, v15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decodark15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECO Cassette System ROM Multigame (Darksoft, v16)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decodark16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECO Cassette System ROM Multigame (Darksoft, v17)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decodark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECO Cassette System ROM Multigame (David Widel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decomult</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disco No.1 (DECO Cassette)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cdiscon1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Controls Don’t Work – Gameplay is Messed up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DS Telejan (DECO Cassette) (Japan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cdsteljn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mahjong panel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needs Different controls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explorer (DECO Cassette) (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cexplore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fighting Ice Hockey (DECO Cassette)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cfghtice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fishing (DECO Cassette) (Japan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cfishing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flash Boy (vertical) (DECO Cassette MD) (No.12/Ver.0/Set.1,Japan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cfboy0a1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flying Ball (DECO Cassette)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cflyball</t>
+  </si>
+  <si>
     <t xml:space="preserve">No</t>
   </si>
   <si>
-    <t xml:space="preserve">Cassette Error #01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Angler Dangler (DECO Cassette) (US)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cadanglr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Astro Fantasia (DECO Cassette) (US)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">castfant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Boulder Dash (DECO Cassette) (US)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cbdash</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bump 'n' Jump (DECO Cassette) (US)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cbnj</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burger Time (DECO Cassette) (US)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cbtime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burnin' Rubber (DECO Cassette) (Japan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cburnrubj</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burnin' Rubber (DECO Cassette)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cburnrub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burnin' Rubber (DECO Cassette) (US) (set 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cburnrub2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster Buster (DECO Cassette) (US)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cgraplop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DECO Cassette System ROM Multigame (Darksoft, v15)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">decodark15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loads, but Yellow Screen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DECO Cassette System ROM Multigame (Darksoft, v16)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">decodark16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DECO Cassette System ROM Multigame (Darksoft, v17)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">decodark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loads, but Requires Soft Reset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DECO Cassette System ROM Multigame (David Widel)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">decomult</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disco No.1 (DECO Cassette)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cdiscon1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Controls Don’t Work – Gameplay is Messed up</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DS Telejan (DECO Cassette) (Japan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cdsteljn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mahjong panel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Needs Different controls</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Explorer (DECO Cassette) (US)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cexplore</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fighting Ice Hockey (DECO Cassette)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cfghtice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fishing (DECO Cassette) (Japan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cfishing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flash Boy (vertical) (DECO Cassette MD) (No.12/Ver.0/Set.1,Japan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cfboy0a1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flying Ball (DECO Cassette)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cflyball</t>
-  </si>
-  <si>
     <t xml:space="preserve">Loads, but Resets End-of-Load</t>
   </si>
   <si>
@@ -416,9 +407,6 @@
   </si>
   <si>
     <t xml:space="preserve">Dual joysticks (left + right stick)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fix the Dual Joysticks</t>
   </si>
   <si>
     <t xml:space="preserve">Tornado (DECO Cassette) (US)</t>
@@ -693,34 +681,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -909,7 +897,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
@@ -920,18 +908,18 @@
         <v>7</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>7</v>
@@ -945,10 +933,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>7</v>
@@ -962,10 +950,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>7</v>
@@ -979,10 +967,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>7</v>
@@ -996,10 +984,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>7</v>
@@ -1013,10 +1001,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>7</v>
@@ -1030,10 +1018,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>7</v>
@@ -1047,10 +1035,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>7</v>
@@ -1064,78 +1052,78 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="C13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B14" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="3" t="s">
+      <c r="C14" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>38</v>
-      </c>
       <c r="C15" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>40</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>7</v>
@@ -1149,44 +1137,44 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>7</v>
@@ -1200,10 +1188,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>7</v>
@@ -1217,10 +1205,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>7</v>
@@ -1234,10 +1222,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>7</v>
@@ -1251,27 +1239,27 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>7</v>
@@ -1285,10 +1273,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>7</v>
@@ -1302,10 +1290,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>7</v>
@@ -1319,10 +1307,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>7</v>
@@ -1336,10 +1324,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>7</v>
@@ -1353,10 +1341,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>7</v>
@@ -1370,10 +1358,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>7</v>
@@ -1387,10 +1375,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>7</v>
@@ -1404,10 +1392,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>7</v>
@@ -1421,10 +1409,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>7</v>
@@ -1438,10 +1426,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>7</v>
@@ -1455,10 +1443,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>7</v>
@@ -1472,13 +1460,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>8</v>
@@ -1489,13 +1477,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>8</v>
@@ -1506,10 +1494,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>7</v>
@@ -1523,10 +1511,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>7</v>
@@ -1540,10 +1528,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>7</v>
@@ -1557,10 +1545,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>7</v>
@@ -1574,10 +1562,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>7</v>
@@ -1591,10 +1579,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>7</v>
@@ -1608,10 +1596,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>7</v>
@@ -1625,10 +1613,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>7</v>
@@ -1642,10 +1630,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>7</v>
@@ -1659,10 +1647,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>7</v>
@@ -1676,10 +1664,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>7</v>
@@ -1693,10 +1681,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>7</v>
@@ -1710,10 +1698,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>7</v>
@@ -1727,10 +1715,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>7</v>
@@ -1744,10 +1732,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>7</v>
@@ -1761,27 +1749,27 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>7</v>
@@ -1795,44 +1783,44 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B56" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="C55" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E55" s="3" t="s">
+      <c r="C56" s="4" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>130</v>
-      </c>
       <c r="D56" s="4" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>131</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>7</v>
@@ -1846,10 +1834,10 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>7</v>
@@ -1863,10 +1851,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>7</v>
@@ -1880,10 +1868,10 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>7</v>
@@ -1897,10 +1885,10 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>7</v>
@@ -1914,10 +1902,10 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>7</v>
@@ -1931,10 +1919,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Updated RBF - Fast Loader (Overclocked Tape) Now Added to OSD
</commit_message>
<xml_diff>
--- a/Useful Information/DECO_Cassette_Test_List.xlsx
+++ b/Useful Information/DECO_Cassette_Test_List.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="137">
   <si>
     <t xml:space="preserve">Game Name</t>
   </si>
@@ -145,12 +145,6 @@
     <t xml:space="preserve">cdiscon1</t>
   </si>
   <si>
-    <t xml:space="preserve">Partial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Controls Don’t Work – Gameplay is Messed up</t>
-  </si>
-  <si>
     <t xml:space="preserve">DS Telejan (DECO Cassette) (Japan)</t>
   </si>
   <si>
@@ -193,12 +187,6 @@
     <t xml:space="preserve">cflyball</t>
   </si>
   <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loads, but Resets End-of-Load</t>
-  </si>
-  <si>
     <t xml:space="preserve">Graplop (DECO Cassette) (Japan)</t>
   </si>
   <si>
@@ -380,9 +368,6 @@
   </si>
   <si>
     <t xml:space="preserve">csweetht</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loads, but Black Screen Sometimes – Unreliable?</t>
   </si>
   <si>
     <t xml:space="preserve">Terranean (DECO Cassette) (US)</t>
@@ -1146,35 +1131,35 @@
         <v>7</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="D18" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>7</v>
@@ -1188,10 +1173,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>7</v>
@@ -1205,10 +1190,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>7</v>
@@ -1222,44 +1207,44 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B23" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>55</v>
-      </c>
       <c r="C23" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>57</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>7</v>
@@ -1273,10 +1258,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>7</v>
@@ -1290,10 +1275,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>7</v>
@@ -1307,10 +1292,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>7</v>
@@ -1324,10 +1309,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>7</v>
@@ -1341,10 +1326,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>7</v>
@@ -1358,10 +1343,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>7</v>
@@ -1375,10 +1360,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>7</v>
@@ -1392,10 +1377,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>7</v>
@@ -1409,10 +1394,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>7</v>
@@ -1426,10 +1411,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>7</v>
@@ -1443,10 +1428,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>7</v>
@@ -1460,13 +1445,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>8</v>
@@ -1477,13 +1462,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>8</v>
@@ -1494,10 +1479,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>7</v>
@@ -1511,10 +1496,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>7</v>
@@ -1528,10 +1513,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>7</v>
@@ -1545,10 +1530,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>7</v>
@@ -1562,10 +1547,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>7</v>
@@ -1579,10 +1564,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>7</v>
@@ -1596,10 +1581,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>7</v>
@@ -1613,10 +1598,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>7</v>
@@ -1630,10 +1615,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>7</v>
@@ -1647,10 +1632,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>7</v>
@@ -1664,10 +1649,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>7</v>
@@ -1681,10 +1666,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>7</v>
@@ -1698,10 +1683,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>7</v>
@@ -1715,10 +1700,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>7</v>
@@ -1732,10 +1717,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>7</v>
@@ -1749,27 +1734,27 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>119</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>7</v>
@@ -1783,10 +1768,10 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>7</v>
@@ -1795,18 +1780,18 @@
         <v>8</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>8</v>
@@ -1817,10 +1802,10 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>7</v>
@@ -1834,10 +1819,10 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>7</v>
@@ -1851,10 +1836,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>7</v>
@@ -1868,10 +1853,10 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>7</v>
@@ -1885,10 +1870,10 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>7</v>
@@ -1902,10 +1887,10 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>7</v>
@@ -1919,10 +1904,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>7</v>

</xml_diff>